<commit_message>
Update board — 0 notes, 0 done (2026-08-18 15:04)
</commit_message>
<xml_diff>
--- a/data/todo-board-Vidya.xlsx
+++ b/data/todo-board-Vidya.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:J2"/>
   <cols>
     <col min="1" max="1" width="11.83203125" customWidth="1"/>
     <col min="2" max="2" width="34.83203125" customWidth="1"/>
@@ -448,103 +448,39 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>T-GTSZ553</v>
+        <v/>
       </c>
       <c r="B2" t="str">
-        <v>Open the Activity log sheet</v>
+        <v/>
       </c>
       <c r="C2" t="str">
-        <v>A dated row for every edit, status change and deletion.</v>
+        <v/>
       </c>
       <c r="D2" t="str">
-        <v>To do</v>
-      </c>
-      <c r="E2">
-        <v>0</v>
+        <v/>
+      </c>
+      <c r="E2" t="str">
+        <v/>
       </c>
       <c r="F2" t="str">
         <v/>
       </c>
       <c r="G2" t="str">
-        <v>2026-08-18</v>
+        <v/>
       </c>
       <c r="H2" t="str">
         <v/>
       </c>
       <c r="I2" t="str">
-        <v>2026-08-18 15:03</v>
+        <v/>
       </c>
       <c r="J2" t="str">
-        <v>--p3</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>T-GTSZ528</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Drag the progress slider</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Reaching 100% marks the note done and stamps the completion date.</v>
-      </c>
-      <c r="D3" t="str">
-        <v>In progress</v>
-      </c>
-      <c r="E3">
-        <v>40</v>
-      </c>
-      <c r="F3" t="str">
-        <v/>
-      </c>
-      <c r="G3" t="str">
-        <v>2026-08-18</v>
-      </c>
-      <c r="H3" t="str">
-        <v/>
-      </c>
-      <c r="I3" t="str">
-        <v>2026-08-18 15:03</v>
-      </c>
-      <c r="J3" t="str">
-        <v>--p2</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>T-GTSZ525</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Welcome to your board</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Write straight onto a note. Everything is stored in the Excel file — no database anywhere.</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Done</v>
-      </c>
-      <c r="E4">
-        <v>100</v>
-      </c>
-      <c r="F4" t="str">
-        <v/>
-      </c>
-      <c r="G4" t="str">
-        <v>2026-08-18</v>
-      </c>
-      <c r="H4" t="str">
-        <v>2026-08-18</v>
-      </c>
-      <c r="I4" t="str">
-        <v>2026-08-18 15:03</v>
-      </c>
-      <c r="J4" t="str">
-        <v>--p1</v>
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J2"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -570,7 +506,7 @@
         <v>Total notes</v>
       </c>
       <c r="B2">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -578,7 +514,7 @@
         <v>To do</v>
       </c>
       <c r="B3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -586,7 +522,7 @@
         <v>In progress</v>
       </c>
       <c r="B4">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -594,7 +530,7 @@
         <v>Done</v>
       </c>
       <c r="B5">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -602,7 +538,7 @@
         <v>Overall progress %</v>
       </c>
       <c r="B6">
-        <v>47</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -618,7 +554,7 @@
         <v>In bin</v>
       </c>
       <c r="B8">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9">
@@ -626,7 +562,7 @@
         <v>Last saved</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-08-18 15:03</v>
+        <v>2026-08-18 15:04</v>
       </c>
     </row>
   </sheetData>
@@ -638,7 +574,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K4"/>
   <cols>
     <col min="1" max="1" width="11.83203125" customWidth="1"/>
     <col min="2" max="2" width="34.83203125" customWidth="1"/>
@@ -690,49 +626,119 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v/>
+        <v>T-GTSZ525</v>
       </c>
       <c r="B2" t="str">
-        <v/>
+        <v>Welcome to your board</v>
       </c>
       <c r="C2" t="str">
-        <v/>
+        <v>Write straight onto a note. Everything is stored in the Excel file — no database anywhere.</v>
       </c>
       <c r="D2" t="str">
-        <v/>
-      </c>
-      <c r="E2" t="str">
-        <v/>
+        <v>Done</v>
+      </c>
+      <c r="E2">
+        <v>100</v>
       </c>
       <c r="F2" t="str">
         <v/>
       </c>
       <c r="G2" t="str">
-        <v/>
+        <v>2026-08-18</v>
       </c>
       <c r="H2" t="str">
-        <v/>
+        <v>2026-08-18</v>
       </c>
       <c r="I2" t="str">
-        <v/>
+        <v>2026-08-18 15:03</v>
       </c>
       <c r="J2" t="str">
-        <v/>
+        <v>--p1</v>
       </c>
       <c r="K2" t="str">
-        <v/>
+        <v>2026-08-18 15:03</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>T-GTSZ528</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Drag the progress slider</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Reaching 100% marks the note done and stamps the completion date.</v>
+      </c>
+      <c r="D3" t="str">
+        <v>In progress</v>
+      </c>
+      <c r="E3">
+        <v>40</v>
+      </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+      <c r="G3" t="str">
+        <v>2026-08-18</v>
+      </c>
+      <c r="H3" t="str">
+        <v/>
+      </c>
+      <c r="I3" t="str">
+        <v>2026-08-18 15:03</v>
+      </c>
+      <c r="J3" t="str">
+        <v>--p2</v>
+      </c>
+      <c r="K3" t="str">
+        <v>2026-08-18 15:03</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>T-GTSZ553</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Open the Activity log sheet</v>
+      </c>
+      <c r="C4" t="str">
+        <v>A dated row for every edit, status change and deletion.</v>
+      </c>
+      <c r="D4" t="str">
+        <v>To do</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4" t="str">
+        <v>2026-08-18</v>
+      </c>
+      <c r="H4" t="str">
+        <v/>
+      </c>
+      <c r="I4" t="str">
+        <v>2026-08-18 15:03</v>
+      </c>
+      <c r="J4" t="str">
+        <v>--p3</v>
+      </c>
+      <c r="K4" t="str">
+        <v>2026-08-18 15:03</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K4"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E7"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -809,9 +815,60 @@
         <v/>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>2026-08-18 15:03</v>
+      </c>
+      <c r="B5" t="str">
+        <v>T-GTSZ553</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Open the Activity log sheet</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Moved to bin</v>
+      </c>
+      <c r="E5" t="str">
+        <v>was To do at 0%</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>2026-08-18 15:03</v>
+      </c>
+      <c r="B6" t="str">
+        <v>T-GTSZ528</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Drag the progress slider</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Moved to bin</v>
+      </c>
+      <c r="E6" t="str">
+        <v>was In progress at 40%</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>2026-08-18 15:03</v>
+      </c>
+      <c r="B7" t="str">
+        <v>T-GTSZ525</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Welcome to your board</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Moved to bin</v>
+      </c>
+      <c r="E7" t="str">
+        <v>was Done at 100%</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>